<commit_message>
upload 4th week codes
</commit_message>
<xml_diff>
--- a/学习资料/React Learning.xlsx
+++ b/学习资料/React Learning.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WorkSpace\react-learning\学习资料\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9480E26-61F8-4A77-86C7-F76B3F24F0F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B62BA1C-1641-4DD0-BCC5-2FBC586938D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{17DF913D-669B-42EF-B225-336789998B9A}"/>
   </bookViews>
@@ -74,9 +74,6 @@
     <t>React 生态与工程化</t>
   </si>
   <si>
-    <t>React Router（路由）、Axios/fetch（请求）Redux（状态管理）、Ant Design/MUI（UI组件库），表单处理（React Hook Form），memo, useMemo, useCallback、代码分割、ESLint/Prettier 规范</t>
-  </si>
-  <si>
     <t>开发一个具备</t>
   </si>
   <si>
@@ -117,13 +114,35 @@
   </si>
   <si>
     <t>用时(周)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>React Router（路由）、Axios/fetch（请求）Redux（状态管理）、Ant Design/MUI（UI组件库），表单处理（React Hook Form），memo, useMemo, useCallback</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>、代码分割、ESLint/Prettier 规范</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -135,6 +154,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -160,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -169,6 +195,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -529,7 +558,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -539,10 +568,10 @@
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="4" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="1">
@@ -556,10 +585,10 @@
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="1">
@@ -574,10 +603,10 @@
         <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="E4" s="3">
         <v>6</v>
@@ -587,8 +616,8 @@
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
-      <c r="D5" s="1" t="s">
-        <v>13</v>
+      <c r="D5" s="4" t="s">
+        <v>12</v>
       </c>
       <c r="E5" s="3"/>
     </row>
@@ -596,8 +625,8 @@
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="1" t="s">
-        <v>14</v>
+      <c r="D6" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="E6" s="3"/>
     </row>
@@ -605,8 +634,8 @@
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="1" t="s">
-        <v>15</v>
+      <c r="D7" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="E7" s="3"/>
     </row>
@@ -614,8 +643,8 @@
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
-      <c r="D8" s="1" t="s">
-        <v>16</v>
+      <c r="D8" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="E8" s="3"/>
     </row>
@@ -623,8 +652,8 @@
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
-      <c r="D9" s="1" t="s">
-        <v>17</v>
+      <c r="D9" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="E9" s="3"/>
     </row>
@@ -632,8 +661,8 @@
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
-      <c r="D10" s="1" t="s">
-        <v>18</v>
+      <c r="D10" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="E10" s="3"/>
     </row>
@@ -642,7 +671,7 @@
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E11" s="3"/>
     </row>
@@ -651,7 +680,7 @@
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E12" s="3"/>
     </row>
@@ -660,7 +689,7 @@
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E13" s="3"/>
     </row>
@@ -669,13 +698,13 @@
         <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="E14" s="1">
         <v>4</v>

</xml_diff>